<commit_message>
Sync the test plan with the repository
- File names (.ts configs and support file, cypress.ci.config.ts)
- Test data lives in Gherkin tables, not fixtures; Chrome is the only
  browser; Cucumber HTML report from the preprocessor; no data-state
- Steps of TC-001, TC-002, TC-004, TC-005, TC-012, TC-013 and TC-015
  match the reworked scenarios
- New "Last run" column with a link to the CI run behind each status
- Summary note describes the COUNTIF formulas precisely
</commit_message>
<xml_diff>
--- a/docs/telnyx-test-plan.xlsx
+++ b/docs/telnyx-test-plan.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$N$16</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Test Cases'!$A$1:$O$16</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="180">
   <si>
     <t xml:space="preserve">Telnyx.com UI Test Plan — Cypress + Cucumber</t>
   </si>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">Version / Date</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0 / 2026-10-22</t>
+    <t xml:space="preserve">1.1 / 2026-10-23</t>
   </si>
   <si>
     <t xml:space="preserve">Objective</t>
@@ -89,16 +89,17 @@
   </si>
   <si>
     <t xml:space="preserve">• BDD: Gherkin .feature files grouped by site area + step definitions
-• Page Object pattern for locators and actions
-• Test data (navigation items, social URLs) in fixtures
-• Tags: @smoke for the critical path, @regression for the full suite
-• Assertions target stable visible content and semantic attributes (href, target, aria-expanded, data-state)</t>
+• Page Object pattern: pages extend BasePage; the site-wide header and footer are separate components
+• Test data (navigation items, social URLs, emails, expected messages) in Gherkin data tables and step parameters
+• Tags: @TC-xxx for each test case, @smoke for the critical path, @regression for the full suite
+• Links are found by their visible text, and the href is asserted separately
+• Assertions target stable visible content and semantic attributes (href, target, aria-expanded)</t>
   </si>
   <si>
     <t xml:space="preserve">Known site behaviour</t>
   </si>
   <si>
-    <t xml:space="preserve">telnyx.com throws its own uncaught errors (document.modelContext SecurityError, cross-origin 'Script error.'). Only these are ignored in cypress/support/e2e.js; any other application error still fails the test. The OneTrust cookie banner is suppressed by setting consent cookies before each test.</t>
+    <t xml:space="preserve">telnyx.com throws its own uncaught errors (document.modelContext SecurityError, cross-origin 'Script error.'). Only these are ignored in cypress/support/e2e.ts; any other application error still fails the test. The OneTrust cookie banner is suppressed by setting consent cookies before each test.</t>
   </si>
   <si>
     <t xml:space="preserve">Environment</t>
@@ -113,25 +114,25 @@
     <t xml:space="preserve">Browsers</t>
   </si>
   <si>
-    <t xml:space="preserve">Chrome (primary, CI), Electron (Cypress default); desktop viewport 1440 × 900, mobile viewport 375 × 812</t>
+    <t xml:space="preserve">Chrome (local runs and CI); desktop viewport 1440 × 900, mobile viewport 375 × 812 (Cypress iphone-x preset)</t>
   </si>
   <si>
     <t xml:space="preserve">Tools</t>
   </si>
   <si>
-    <t xml:space="preserve">Node.js LTS, Cypress, @badeball/cypress-cucumber-preprocessor, esbuild, HTML report (cucumber/mochawesome), GitHub Actions, GitHub Pages</t>
+    <t xml:space="preserve">Node.js 24, Cypress, TypeScript, @badeball/cypress-cucumber-preprocessor, esbuild, Cucumber HTML report (built into the preprocessor), ESLint + Prettier, GitHub Actions, GitHub Pages</t>
   </si>
   <si>
     <t xml:space="preserve">Configuration</t>
   </si>
   <si>
-    <t xml:space="preserve">Base config cypress.config.js plus a separate environment config file (e.g. cypress.prod.config.js) selected with --config-file; base URL configurable.</t>
+    <t xml:space="preserve">Base config cypress.config.ts for local runs (no retries) plus cypress.ci.config.ts for GitHub Actions (longer timeouts, 2 retries), selected with --config-file.</t>
   </si>
   <si>
     <t xml:space="preserve">CI / Reporting</t>
   </si>
   <si>
-    <t xml:space="preserve">GitHub Actions runs the suite on push / pull request / manual trigger, uploads screenshots on failure, generates an HTML report and publishes it to GitHub Pages.</t>
+    <t xml:space="preserve">GitHub Actions runs on push to main, pull requests and manual trigger: type check, lint, format check, tests. Screenshots and the HTML report are uploaded as artifacts on every run; on main the report is published to GitHub Pages.</t>
   </si>
   <si>
     <t xml:space="preserve">Criteria</t>
@@ -210,6 +211,9 @@
     <t xml:space="preserve">Comments</t>
   </si>
   <si>
+    <t xml:space="preserve">Last run</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-001</t>
   </si>
   <si>
@@ -237,10 +241,11 @@
     <t xml:space="preserve">URL: https://telnyx.com/</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open https://telnyx.com/.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The homepage loads and the browser URL is https://telnyx.com/.</t>
+    <t xml:space="preserve">1. Open https://telnyx.com/.
+2. Check the URL, the site header and the main heading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The browser URL is https://telnyx.com/ and the site header and the main heading are displayed.</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
@@ -249,10 +254,13 @@
     <t xml:space="preserve">Passed</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-22, CI run #1</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-002</t>
   </si>
   <si>
-    <t xml:space="preserve">Verify logo is visible and navigates to homepage</t>
+    <t xml:space="preserve">Verify logo navigates to homepage</t>
   </si>
   <si>
     <t xml:space="preserve">Medium</t>
@@ -264,18 +272,18 @@
     <t xml:space="preserve">@regression</t>
   </si>
   <si>
-    <t xml:space="preserve">Homepage is open; cookie banner is suppressed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logo link href: /</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Locate the Telnyx logo in the site header.
-2. Verify it is visible and links to '/'.
+    <t xml:space="preserve">Pricing page is open; cookie banner is suppressed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start page: /pricing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open https://telnyx.com/pricing.
+2. Verify the Telnyx logo is visible in the site header.
 3. Click the logo.</t>
   </si>
   <si>
-    <t xml:space="preserve">The logo is visible, has the homepage link, and clicking it opens https://telnyx.com/.</t>
+    <t xml:space="preserve">Clicking the logo opens https://telnyx.com/ with the site header and the main heading displayed.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-003</t>
@@ -321,15 +329,19 @@
     <t xml:space="preserve">Navigation</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected URL part: /sign-up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Click the Sign up link in the header.
-2. Wait for the registration page to load.
+    <t xml:space="preserve">Homepage is open; cookie banner is suppressed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected href: /sign-up
+Expected heading: Create your account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Find the Sign up link in the header by its text and check its href.
+2. Click the link.
 3. Check the page URL and heading.</t>
   </si>
   <si>
-    <t xml:space="preserve">The URL contains '/sign-up' and the 'Create your account' heading is displayed.</t>
+    <t xml:space="preserve">The link points to /sign-up, the URL contains '/sign-up' and the 'Create your account' heading is displayed.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-005</t>
@@ -341,7 +353,7 @@
     <t xml:space="preserve">Expected href: https://portal.telnyx.com</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Verify the Log in link is visible and points to https://portal.telnyx.com.
+    <t xml:space="preserve">1. Find the Log in link in the header by its text; verify it is visible and points to https://portal.telnyx.com.
 2. Click the link (opened in the same tab for the test).
 3. Verify the portal sign-in page opens.</t>
   </si>
@@ -498,15 +510,15 @@
     <t xml:space="preserve">Verify mobile navigation menu opens</t>
   </si>
   <si>
-    <t xml:space="preserve">Viewport is set to 375 × 812; homepage is open; cookie banner is suppressed.</t>
+    <t xml:space="preserve">Viewport is set to 375 × 812 (iphone-x); homepage is open; cookie banner is suppressed.</t>
   </si>
   <si>
     <t xml:space="preserve">Viewport: 375 × 812</t>
   </si>
   <si>
     <t xml:space="preserve">1. Open the homepage at mobile viewport size.
-2. Locate the mobile menu button.
-3. Click the button.
+2. Verify the mobile menu button is visible and the menu is closed.
+3. Open the mobile menu.
 4. Verify the navigation menu is open.</t>
   </si>
   <si>
@@ -525,10 +537,9 @@
     <t xml:space="preserve">Dropdowns: Products, Solutions</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Open the Products dropdown.
-2. Verify it is expanded.
-3. Open the Solutions dropdown.
-4. Check the expanded state of both dropdowns.</t>
+    <t xml:space="preserve">1. Open the Products dropdown and verify it is expanded.
+2. Open the Solutions dropdown.
+3. Check the expanded state of both dropdowns.</t>
   </si>
   <si>
     <t xml:space="preserve">Solutions has aria-expanded='true' and Products has aria-expanded='false'.</t>
@@ -575,8 +586,8 @@
 Terms checkbox: checked</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Enter an invalid email.
-2. Accept the terms checkbox to isolate email validation.
+    <t xml:space="preserve">1. Accept the terms checkbox to isolate email validation.
+2. Enter an invalid email.
 3. Click Create account.
 4. Inspect the email validation message.</t>
   </si>
@@ -587,7 +598,7 @@
     <t xml:space="preserve">Test Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Counts update automatically from the Status column on the Test Cases sheet.</t>
+    <t xml:space="preserve">Counts are COUNTIF formulas over the Priority, Area and Status columns of the Test Cases sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Test cases</t>
@@ -616,7 +627,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -672,6 +683,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -775,16 +794,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -804,11 +827,15 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -825,7 +852,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -877,6 +904,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0563C1"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -948,7 +983,7 @@
       <rgbColor rgb="FFFFE699"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -999,34 +1034,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1037,69 +1072,11 @@
         <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1230,193 +1207,193 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="110"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+    <row r="18" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+      <c r="B25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1446,718 +1423,767 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="N1" s="6" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="4" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="G2" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="K2" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="L2" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="N2" s="4"/>
-    </row>
-    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+      <c r="M2" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="N2" s="5"/>
+      <c r="O2" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N3" s="5"/>
+      <c r="O3" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="G3" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N4" s="5"/>
+      <c r="O4" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N5" s="5"/>
+      <c r="O5" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N6" s="5"/>
+      <c r="O6" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N7" s="5"/>
+      <c r="O7" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N8" s="5"/>
+      <c r="O8" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I3" s="4" t="s">
+      <c r="F9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" s="6" t="s">
+      <c r="H9" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L9" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="N3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="M9" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N9" s="5"/>
+      <c r="O9" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N10" s="5"/>
+      <c r="O10" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" s="5"/>
+      <c r="O11" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M12" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N12" s="5"/>
+      <c r="O12" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="M13" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N13" s="5"/>
+      <c r="O13" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M4" s="6" t="s">
+      <c r="D14" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="L14" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="N4" s="4"/>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M5" s="6" t="s">
+      <c r="M14" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N14" s="5"/>
+      <c r="O14" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="L15" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="N5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M6" s="6" t="s">
+      <c r="M15" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N15" s="5"/>
+      <c r="O15" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="L16" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="N6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N7" s="4"/>
-    </row>
-    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N8" s="4"/>
-    </row>
-    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N9" s="4"/>
-    </row>
-    <row r="10" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M10" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N10" s="4"/>
-    </row>
-    <row r="11" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M11" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N11" s="4"/>
-    </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="L12" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M12" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N12" s="4"/>
-    </row>
-    <row r="13" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N13" s="4"/>
-    </row>
-    <row r="14" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M14" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N14" s="4"/>
-    </row>
-    <row r="15" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="J15" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="N16" s="4"/>
+      <c r="M16" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="N16" s="5"/>
+      <c r="O16" s="8" t="s">
+        <v>69</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N16"/>
+  <autoFilter ref="A1:O16"/>
   <conditionalFormatting sqref="E2:E16">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>"Medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M16">
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"Passed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Failed"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2167,6 +2193,23 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="O2" r:id="rId1" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O3" r:id="rId2" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O4" r:id="rId3" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O5" r:id="rId4" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O6" r:id="rId5" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O7" r:id="rId6" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O8" r:id="rId7" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O9" r:id="rId8" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O10" r:id="rId9" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O11" r:id="rId10" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O12" r:id="rId11" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O13" r:id="rId12" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O14" r:id="rId13" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O15" r:id="rId14" display="2026-10-22, CI run #1"/>
+    <hyperlink ref="O16" r:id="rId15" display="2026-10-22, CI run #1"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2174,7 +2217,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
 
@@ -2184,204 +2227,204 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="4" t="n">
+      <c r="B4" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$E$2:$E$16,A5)</f>
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B6" s="4" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$E$2:$E$16,A6)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B7" s="4" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$E$2:$E$16,A7)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B8" s="3" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" s="4" t="n">
         <f aca="false">SUM(B5:B7)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="4" t="n">
+      <c r="B10" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A11)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="4" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A12)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="B13" s="4" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A13)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B14" s="4" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A14)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B15" s="4" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A15)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="B16" s="4" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="B16" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A16)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="B17" s="4" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B17" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$C$2:$C$16,A17)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B18" s="3" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18" s="4" t="n">
         <f aca="false">SUM(B11:B17)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B21" s="4" t="n">
+      <c r="B20" s="6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="B21" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$M$2:$M$16,A21)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="4" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$M$2:$M$16,A22)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="4" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B23" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$M$2:$M$16,A23)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B24" s="4" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24" s="5" t="n">
         <f aca="false">COUNTIF('Test Cases'!$M$2:$M$16,A24)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B25" s="3" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" s="4" t="n">
         <f aca="false">SUM(B21:B24)</f>
         <v>15</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B27" s="9" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="11" t="n">
         <f aca="false">IFERROR(COUNTIF('Test Cases'!$M$2:$M$16,"Passed")/COUNTA('Test Cases'!$A$2:$A$16),0)</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Update TC-006 in the test plan
The scenario now checks the href of the View all pricing link and the
text of the pricing page heading, so the test data, steps and expected
result describe both.
</commit_message>
<xml_diff>
--- a/docs/telnyx-test-plan.xlsx
+++ b/docs/telnyx-test-plan.xlsx
@@ -376,15 +376,17 @@
     <t xml:space="preserve">Homepage is open in desktop viewport; cookie banner is suppressed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected URL part: /pricing</t>
+    <t xml:space="preserve">Expected href: /pricing
+Expected heading: Pay for what you use</t>
   </si>
   <si>
     <t xml:space="preserve">1. Open the Pricing menu in the header.
-2. Click the link to view all pricing.
-3. Verify the URL and page content.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The browser navigates to '/pricing' and the pricing page content is displayed.</t>
+2. Find the View all pricing link by its text and check its href.
+3. Click the link.
+4. Check the page URL and heading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The link points to /pricing, the URL contains '/pricing' and the 'Pay for what you use.' heading is displayed.</t>
   </si>
   <si>
     <t xml:space="preserve">TC-007</t>

</xml_diff>